<commit_message>
mise en place le telechargement des fichiers excel
</commit_message>
<xml_diff>
--- a/Login_list_for_funds.xlsx
+++ b/Login_list_for_funds.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30023"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aaitmoussa\Desktop\Projet Aplitec\Automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aplitecgroupe.sharepoint.com/sites/Equipes59/Documents partages/Dossiers EC/- 1 Suivi fonds expertise/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4888E3A6-6783-437C-8F14-B2515C31DC66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="11_E9CBE4569E8DD7670001D27560E0DE641A07A215" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{448A5C5A-C93F-4FF3-A972-70735F531E1D}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="35865" yWindow="2730" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="108">
   <si>
     <t>Portail internet Dépositaire</t>
   </si>
@@ -86,6 +86,9 @@
     <t>Aplitec2025?14</t>
   </si>
   <si>
+    <t>julie.malidor@groupe-aplitec.com</t>
+  </si>
+  <si>
     <t>Aldebaran</t>
   </si>
   <si>
@@ -107,6 +110,9 @@
     <t>02AplItEc_425,8</t>
   </si>
   <si>
+    <t>sami.melakhessou@groupe-aplitec.com</t>
+  </si>
+  <si>
     <t>Atalante Equity</t>
   </si>
   <si>
@@ -122,7 +128,7 @@
     <t>7980/ebelloche</t>
   </si>
   <si>
-    <t>APLitec*Ferr@us_4</t>
+    <t>APLitec*Ferr@us_5</t>
   </si>
   <si>
     <t>Activa</t>
@@ -197,6 +203,9 @@
     <t>Aplitec&amp;2025**!a</t>
   </si>
   <si>
+    <t>bruno.dechance@groupe-aplitec.com</t>
+  </si>
+  <si>
     <t>Demeter</t>
   </si>
   <si>
@@ -300,6 +309,12 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Oneragtime</t>
+  </si>
+  <si>
+    <t>12315/abouzeboudja</t>
   </si>
   <si>
     <t>Phitrust</t>
@@ -351,7 +366,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -363,7 +378,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -375,17 +389,22 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -393,21 +412,24 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF242424"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -454,71 +476,58 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="20" fontId="1" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="1" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -540,9 +549,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -580,7 +589,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -686,7 +695,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -828,7 +837,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -836,645 +845,677 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="29.6640625" customWidth="1"/>
-    <col min="2" max="2" width="31.109375" customWidth="1"/>
-    <col min="3" max="3" width="37.5546875" customWidth="1"/>
+    <col min="1" max="1" width="45.85546875" customWidth="1"/>
+    <col min="2" max="2" width="31.140625" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="5" width="36.109375" customWidth="1"/>
-    <col min="6" max="6" width="39.5546875" customWidth="1"/>
+    <col min="5" max="5" width="36.140625" customWidth="1"/>
+    <col min="6" max="6" width="43.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="15.75">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="24"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="3"/>
-    </row>
-    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="D1" s="2"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="4"/>
+    </row>
+    <row r="2" spans="1:6" ht="15.75">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:6" ht="15.75">
+      <c r="A3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:6" ht="15.75">
+      <c r="A4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="10" t="s">
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="F4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="2" t="s">
+    </row>
+    <row r="5" spans="1:6" ht="15.75">
+      <c r="A5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>17</v>
+      <c r="D5" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="F5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="7" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="15.75">
+      <c r="A6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="E6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="7" t="s">
+      <c r="F6" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.75">
+      <c r="A7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:6" ht="15.75">
+      <c r="A8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75">
+      <c r="A9" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.75">
+      <c r="A10" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.75">
+      <c r="A11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.75">
+      <c r="A12" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="15.75">
+      <c r="A13" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="15.75">
+      <c r="A14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D14" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" s="7" t="s">
+      <c r="E14" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F10" s="3" t="s">
+    <row r="15" spans="1:6" ht="15.75">
+      <c r="A15" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="15.75">
+      <c r="A16" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="15.75">
+      <c r="A17" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15.75">
+      <c r="A18" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.75">
+      <c r="A19" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15.75">
+      <c r="A20" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="15.75">
+      <c r="A21" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="15.75">
+      <c r="A22" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="15.75">
+      <c r="A23" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="15.75">
+      <c r="A24" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E24" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15.75">
+      <c r="A25" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="15.75">
+      <c r="A26" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="F26" s="12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="10" t="s">
+    <row r="27" spans="1:6" ht="15.75">
+      <c r="A27" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F27" s="4"/>
+    </row>
+    <row r="28" spans="1:6" ht="15.75">
+      <c r="A28" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="19" t="s">
+      <c r="F28" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15.75">
+      <c r="A29" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
+      <c r="C29" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D29" s="3">
+        <v>40671265</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="F29" s="4"/>
+    </row>
+    <row r="30" spans="1:6" ht="15.75">
+      <c r="A30" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="15.75">
+      <c r="A31" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="D31" s="3">
+        <v>40706895</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="F31" s="4"/>
+    </row>
+    <row r="32" spans="1:6" ht="15.75">
+      <c r="A32" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C32" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E15" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" s="3"/>
-    </row>
-    <row r="16" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="E16" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="E18" s="2" t="s">
+      <c r="D32" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F32" s="4"/>
+    </row>
+    <row r="33" spans="1:6" ht="15.75">
+      <c r="A33" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="15.75">
+      <c r="A34" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F19" s="3"/>
-    </row>
-    <row r="20" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="F23" s="3"/>
-    </row>
-    <row r="24" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B26" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="E26" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="F26" s="3"/>
-    </row>
-    <row r="27" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="F27" s="3"/>
-    </row>
-    <row r="28" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="D28" s="10">
-        <v>40671265</v>
-      </c>
-      <c r="E28" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="F28" s="3"/>
-    </row>
-    <row r="29" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C30" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="D30" s="10">
-        <v>40706895</v>
-      </c>
-      <c r="E30" s="19" t="s">
-        <v>96</v>
-      </c>
-      <c r="F30" s="3"/>
-    </row>
-    <row r="31" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="F31" s="3"/>
-    </row>
-    <row r="32" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="B32" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>19</v>
+      <c r="F34" s="4" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1483,18 +1524,18 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{42F8301F-632C-4770-87CB-4563FD9C493E}"/>
-    <hyperlink ref="C28" r:id="rId2" xr:uid="{4A3C22E0-3060-448C-B481-305B7AB53A0F}"/>
+    <hyperlink ref="C29" r:id="rId2" xr:uid="{4A3C22E0-3060-448C-B481-305B7AB53A0F}"/>
     <hyperlink ref="E5" r:id="rId3" display="Aldebaran#2022@" xr:uid="{D6D7D1AF-FC17-47E2-9FE5-6A29FEEDBC1E}"/>
     <hyperlink ref="C23" r:id="rId4" xr:uid="{D06DA950-83DD-46D3-8877-303D43920B9D}"/>
-    <hyperlink ref="E28" r:id="rId5" xr:uid="{30A47FFE-068C-4A64-ADE0-14AEBD63690F}"/>
+    <hyperlink ref="E29" r:id="rId5" xr:uid="{30A47FFE-068C-4A64-ADE0-14AEBD63690F}"/>
     <hyperlink ref="C5" r:id="rId6" xr:uid="{D7C249BA-6678-44E7-95FE-01D31C1A2753}"/>
     <hyperlink ref="C3" r:id="rId7" xr:uid="{33AAFFFD-F227-4BAD-AAE1-7AE8A98BE566}"/>
     <hyperlink ref="C14" r:id="rId8" xr:uid="{875982AD-9F80-4F1F-8A64-A71A4CB86D3F}"/>
     <hyperlink ref="C15" r:id="rId9" xr:uid="{30A16087-01D5-469D-9FBD-3A4E784B1E2E}"/>
     <hyperlink ref="C27" r:id="rId10" xr:uid="{EAD01EFF-1783-43B8-8FA8-5C99D24B543D}"/>
-    <hyperlink ref="E30" r:id="rId11" display="AplitecD23@*+" xr:uid="{77EA1B23-5868-48F9-A79A-03B46C6F4D78}"/>
+    <hyperlink ref="E31" r:id="rId11" display="AplitecD23@*+" xr:uid="{77EA1B23-5868-48F9-A79A-03B46C6F4D78}"/>
     <hyperlink ref="E14" r:id="rId12" xr:uid="{FE8A63B2-9D86-420A-A04C-A4072DD08E01}"/>
-    <hyperlink ref="C32" r:id="rId13" xr:uid="{DA37B202-87C6-4C03-9B23-F27A2924661F}"/>
+    <hyperlink ref="C33" r:id="rId13" xr:uid="{DA37B202-87C6-4C03-9B23-F27A2924661F}"/>
     <hyperlink ref="C7" r:id="rId14" xr:uid="{57EE69CD-EA20-4B03-A0DA-ECB5E07F7D3F}"/>
     <hyperlink ref="C9" r:id="rId15" xr:uid="{05B2B2E2-80DD-41A2-B011-45A2D277142C}"/>
     <hyperlink ref="C13" r:id="rId16" xr:uid="{B8776054-F3F6-43F0-A997-20E1ED59E5C7}"/>
@@ -1503,38 +1544,61 @@
     <hyperlink ref="C10" r:id="rId19" xr:uid="{A27A078E-9083-47DA-B900-82793B48459B}"/>
     <hyperlink ref="C17" r:id="rId20" xr:uid="{AA197180-35F6-454C-95B2-8FFA9E7072FB}"/>
     <hyperlink ref="C20" r:id="rId21" xr:uid="{3E2E36D9-3A7E-4187-BC07-CB31B4635E27}"/>
-    <hyperlink ref="C33" r:id="rId22" xr:uid="{3C7166AA-FAA2-402C-B4ED-2DD7C941FCFA}"/>
+    <hyperlink ref="C34" r:id="rId22" xr:uid="{3C7166AA-FAA2-402C-B4ED-2DD7C941FCFA}"/>
     <hyperlink ref="C12" r:id="rId23" xr:uid="{9B970EF2-1C46-40F9-8A8C-72622F6166F8}"/>
     <hyperlink ref="C16" r:id="rId24" xr:uid="{A48F1953-300E-4550-83C2-CE7900764291}"/>
     <hyperlink ref="C21" r:id="rId25" xr:uid="{9FE6FBD3-E7CA-476B-8B48-1F6788B331D3}"/>
     <hyperlink ref="C6" r:id="rId26" xr:uid="{B0DAEA06-0C63-4C76-83E3-A02E5FB0864B}"/>
     <hyperlink ref="D6" r:id="rId27" display="mailto:pierre@alven.co" xr:uid="{75FE4A90-1848-4DBA-82A7-9DD6ED3D885E}"/>
     <hyperlink ref="D9" r:id="rId28" display="https://www.olisnet.com/OlisAuthenticate/JSP/login.jsp" xr:uid="{30DBB307-0B52-4093-A3C6-D4E3236A3212}"/>
-    <hyperlink ref="C29" r:id="rId29" xr:uid="{C70DBF6E-4593-4F1A-B6A8-AF17602EA718}"/>
+    <hyperlink ref="C30" r:id="rId29" xr:uid="{C70DBF6E-4593-4F1A-B6A8-AF17602EA718}"/>
     <hyperlink ref="C22" r:id="rId30" xr:uid="{DE741FDD-40A3-4055-BC72-E3CF35D7CFED}"/>
     <hyperlink ref="C24" r:id="rId31" xr:uid="{FD5B3648-5992-4B2A-9FF1-3E6C0D8B3644}"/>
     <hyperlink ref="E4" r:id="rId32" display="Aplitec2022@+!!!" xr:uid="{02BA0E5B-9325-42A6-96BF-8A5B51CF1FB6}"/>
     <hyperlink ref="C11" r:id="rId33" xr:uid="{72D1E824-6227-455A-88C4-120844649AFD}"/>
     <hyperlink ref="C8" r:id="rId34" xr:uid="{4422652B-78BB-47B2-A39E-409A84AF6A63}"/>
     <hyperlink ref="E26" r:id="rId35" xr:uid="{EAF9EEF1-D073-4821-A095-76924F9CFFB8}"/>
-    <hyperlink ref="C31" r:id="rId36" xr:uid="{A492A7F2-3ACF-44AD-9BEF-B4D3299BF534}"/>
-    <hyperlink ref="C30" r:id="rId37" xr:uid="{96E36FF5-BE44-4151-85C9-667C3775DBE2}"/>
-    <hyperlink ref="E8" r:id="rId38" xr:uid="{0CC07A86-FFA0-49D2-B324-02A35D6C9795}"/>
-    <hyperlink ref="C25" r:id="rId39" xr:uid="{20B38E72-E1F9-4E65-AF41-73B7A409C74F}"/>
-    <hyperlink ref="C19" r:id="rId40" xr:uid="{80885FD1-AB42-42C7-BA83-59396B563D08}"/>
-    <hyperlink ref="E3" r:id="rId41" xr:uid="{F08359CD-2D3A-4CB7-AF2E-4F2D9E4DE9E1}"/>
-    <hyperlink ref="F3" r:id="rId42" xr:uid="{4132E0CC-3C00-468C-A19B-84F6817EFE2C}"/>
-    <hyperlink ref="F7" r:id="rId43" xr:uid="{992A7E63-972F-4392-BA58-474D8EE418D0}"/>
-    <hyperlink ref="F8" r:id="rId44" xr:uid="{C30E6A9A-3D3A-4DFB-8921-28C299FC89BC}"/>
-    <hyperlink ref="F9" r:id="rId45" xr:uid="{3649B7DF-47A3-4DF1-8ABA-040A0BE8F600}"/>
-    <hyperlink ref="F12" r:id="rId46" xr:uid="{587F1022-A5FD-4171-B4E0-3B7F4B042D17}"/>
+    <hyperlink ref="C32" r:id="rId36" xr:uid="{A492A7F2-3ACF-44AD-9BEF-B4D3299BF534}"/>
+    <hyperlink ref="C31" r:id="rId37" xr:uid="{96E36FF5-BE44-4151-85C9-667C3775DBE2}"/>
+    <hyperlink ref="C25" r:id="rId38" xr:uid="{20B38E72-E1F9-4E65-AF41-73B7A409C74F}"/>
+    <hyperlink ref="C19" r:id="rId39" xr:uid="{80885FD1-AB42-42C7-BA83-59396B563D08}"/>
+    <hyperlink ref="E3" r:id="rId40" xr:uid="{F08359CD-2D3A-4CB7-AF2E-4F2D9E4DE9E1}"/>
+    <hyperlink ref="F3" r:id="rId41" xr:uid="{4132E0CC-3C00-468C-A19B-84F6817EFE2C}"/>
+    <hyperlink ref="F7" r:id="rId42" xr:uid="{992A7E63-972F-4392-BA58-474D8EE418D0}"/>
+    <hyperlink ref="F8" r:id="rId43" xr:uid="{C30E6A9A-3D3A-4DFB-8921-28C299FC89BC}"/>
+    <hyperlink ref="F9" r:id="rId44" xr:uid="{3649B7DF-47A3-4DF1-8ABA-040A0BE8F600}"/>
+    <hyperlink ref="F12" r:id="rId45" xr:uid="{587F1022-A5FD-4171-B4E0-3B7F4B042D17}"/>
+    <hyperlink ref="C28" r:id="rId46" xr:uid="{447ED326-1E3B-447C-85FD-0F918BAB1B80}"/>
+    <hyperlink ref="E8" r:id="rId47" xr:uid="{839C9E81-99C9-4258-9956-7BACA7EEED1E}"/>
+    <hyperlink ref="F23" r:id="rId48" xr:uid="{D0C75622-450A-4D90-AB59-6FB6779810DC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId47"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2bf2f11d-43ed-4181-9932-6864ad410d8c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="37218ea9-0b75-4012-92b8-01d003596ee9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DB89F1DA1EC8B54CA0AF11F05F4C765F" ma:contentTypeVersion="21" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d736f79be593caae3a112933c791ad4e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="2bf2f11d-43ed-4181-9932-6864ad410d8c" xmlns:ns3="37218ea9-0b75-4012-92b8-01d003596ee9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8ae82a03b216e9885234b242cf0adffc" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1812,64 +1876,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2bf2f11d-43ed-4181-9932-6864ad410d8c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="37218ea9-0b75-4012-92b8-01d003596ee9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C731B5DA-5FEE-4470-9C25-3ABA156B7306}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="2bf2f11d-43ed-4181-9932-6864ad410d8c"/>
-    <ds:schemaRef ds:uri="37218ea9-0b75-4012-92b8-01d003596ee9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24D2FF2E-AF41-4DED-B5A8-12232E4A7D1D}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24D2FF2E-AF41-4DED-B5A8-12232E4A7D1D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D748751E-D8B0-4FD4-A4EA-15F59392615D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D748751E-D8B0-4FD4-A4EA-15F59392615D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="2bf2f11d-43ed-4181-9932-6864ad410d8c"/>
-    <ds:schemaRef ds:uri="37218ea9-0b75-4012-92b8-01d003596ee9"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C731B5DA-5FEE-4470-9C25-3ABA156B7306}"/>
 </file>
</xml_diff>